<commit_message>
EX4C Pushed to the website
</commit_message>
<xml_diff>
--- a/week-01/Ex4B_more_GTrends.xlsx
+++ b/week-01/Ex4B_more_GTrends.xlsx
@@ -8,18 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jordan's River\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36EAAACB-2991-4E97-819A-1D5F7EE6EDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{21A306AE-2C60-4CA2-8B81-73C4AC532051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6169690F-3806-41A9-A7C2-2E786527A431}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6169690F-3806-41A9-A7C2-2E786527A431}"/>
   </bookViews>
   <sheets>
     <sheet name="by search term" sheetId="1" r:id="rId1"/>
     <sheet name="by state" sheetId="2" r:id="rId2"/>
+    <sheet name="sales region lookup" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'by search term'!$A$1:$E$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId4"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="67">
   <si>
     <t>Region</t>
   </si>
@@ -211,6 +215,33 @@
   </si>
   <si>
     <t>Breakup</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Sales Region</t>
+  </si>
+  <si>
+    <t>Northwest</t>
+  </si>
+  <si>
+    <t>North Central</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of Hamburger</t>
+  </si>
+  <si>
+    <t>Sum of Milkshake</t>
+  </si>
+  <si>
+    <t>(All)</t>
   </si>
 </sst>
 </file>
@@ -656,7 +687,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -699,13 +730,19 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="42" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -745,6 +782,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Percent" xfId="42" builtinId="5"/>
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
@@ -760,6 +798,1385 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Ex4B_more_GTrends.xlsx]sales region lookup!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'sales region lookup'!$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Hamburger</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'sales region lookup'!$A$16:$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Idaho</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Michigan</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Minnesota</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Montana</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Nebraska</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>North Dakota</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Oregon</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>South Dakota</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Washington</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Wisconsin</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'sales region lookup'!$B$16:$B$26</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.66</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.71</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.69</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.76</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.66</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F178-4330-AFF6-7AD867629EE1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'sales region lookup'!$C$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of Milkshake</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'sales region lookup'!$A$16:$A$26</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Idaho</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Michigan</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Minnesota</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Montana</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Nebraska</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>North Dakota</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Oregon</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>South Dakota</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Washington</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Wisconsin</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'sales region lookup'!$C$16:$C$26</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>0.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.17</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.18</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.14000000000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.19</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F178-4330-AFF6-7AD867629EE1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="780780559"/>
+        <c:axId val="780781039"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="780780559"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="780781039"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="780781039"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="780780559"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>566737</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>261937</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CBC3178F-81D5-78A1-0853-B62838EF5E9E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jordan's River" refreshedDate="46125.890570254633" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{6908C85E-B730-436D-924D-08BB41367F5F}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:D11" sheet="sales region lookup"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="State" numFmtId="0">
+      <sharedItems count="10">
+        <s v="Washington"/>
+        <s v="Oregon"/>
+        <s v="Idaho"/>
+        <s v="Montana"/>
+        <s v="North Dakota"/>
+        <s v="South Dakota"/>
+        <s v="Nebraska"/>
+        <s v="Minnesota"/>
+        <s v="Wisconsin"/>
+        <s v="Michigan"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Sales Region" numFmtId="0">
+      <sharedItems count="2">
+        <s v="Northwest"/>
+        <s v="North Central"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Hamburger" numFmtId="9">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.66" maxValue="0.76"/>
+    </cacheField>
+    <cacheField name="Milkshake" numFmtId="9">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.14000000000000001" maxValue="0.21"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="0.67"/>
+    <n v="0.19"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="0.68"/>
+    <n v="0.18"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="0.67"/>
+    <n v="0.2"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="0.75"/>
+    <n v="0.14000000000000001"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="1"/>
+    <n v="0.69"/>
+    <n v="0.19"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="1"/>
+    <n v="0.76"/>
+    <n v="0.14000000000000001"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <x v="1"/>
+    <n v="0.71"/>
+    <n v="0.17"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <x v="1"/>
+    <n v="0.67"/>
+    <n v="0.19"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <x v="1"/>
+    <n v="0.66"/>
+    <n v="0.2"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <x v="1"/>
+    <n v="0.66"/>
+    <n v="0.21"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6B919F21-F29F-427B-8885-28823D537E34}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A15:C26" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="11">
+        <item x="2"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="9" showAll="0"/>
+    <pivotField dataField="1" numFmtId="9" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="1" hier="-1"/>
+  </pageFields>
+  <dataFields count="2">
+    <dataField name="Sum of Hamburger" fld="2" baseField="0" baseItem="0" numFmtId="9"/>
+    <dataField name="Sum of Milkshake" fld="3" baseField="0" baseItem="0" numFmtId="9"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1098,10 +2515,10 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
         <v>55</v>
-      </c>
-      <c r="D1" t="s">
-        <v>56</v>
       </c>
       <c r="E1" t="s">
         <v>57</v>
@@ -1126,13 +2543,13 @@
         <v>3</v>
       </c>
       <c r="C2" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="D2" s="1">
         <v>0.23</v>
       </c>
-      <c r="D2" s="1">
-        <v>0.68</v>
-      </c>
       <c r="E2" s="1">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1143,13 +2560,13 @@
         <v>35</v>
       </c>
       <c r="C3" s="1">
-        <v>0.16</v>
+        <v>0.72</v>
       </c>
       <c r="D3" s="1">
-        <v>0.64</v>
+        <v>0.15</v>
       </c>
       <c r="E3" s="1">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1160,13 +2577,13 @@
         <v>20</v>
       </c>
       <c r="C4" s="1">
-        <v>0.19</v>
+        <v>0.67</v>
       </c>
       <c r="D4" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="E4" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1177,10 +2594,10 @@
         <v>29</v>
       </c>
       <c r="C5" s="1">
-        <v>0.15</v>
+        <v>0.67</v>
       </c>
       <c r="D5" s="1">
-        <v>0.73</v>
+        <v>0.21</v>
       </c>
       <c r="E5" s="1">
         <v>0.12</v>
@@ -1194,13 +2611,13 @@
         <v>37</v>
       </c>
       <c r="C6" s="1">
-        <v>0.21</v>
+        <v>0.62</v>
       </c>
       <c r="D6" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.2</v>
       </c>
       <c r="E6" s="1">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1211,13 +2628,13 @@
         <v>34</v>
       </c>
       <c r="C7" s="1">
-        <v>0.16</v>
+        <v>0.68</v>
       </c>
       <c r="D7" s="1">
-        <v>0.67</v>
+        <v>0.18</v>
       </c>
       <c r="E7" s="1">
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1228,13 +2645,13 @@
         <v>27</v>
       </c>
       <c r="C8" s="1">
-        <v>0.24</v>
+        <v>0.65</v>
       </c>
       <c r="D8" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.21</v>
       </c>
       <c r="E8" s="1">
-        <v>0.21</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1245,13 +2662,13 @@
         <v>11</v>
       </c>
       <c r="C9" s="1">
-        <v>0.3</v>
+        <v>0.62</v>
       </c>
       <c r="D9" s="1">
-        <v>0.51</v>
+        <v>0.25</v>
       </c>
       <c r="E9" s="1">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1262,13 +2679,13 @@
         <v>24</v>
       </c>
       <c r="C10" s="1">
-        <v>0.27</v>
+        <v>0.67</v>
       </c>
       <c r="D10" s="1">
-        <v>0.41</v>
+        <v>0.17</v>
       </c>
       <c r="E10" s="1">
-        <v>0.32</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1279,13 +2696,13 @@
         <v>13</v>
       </c>
       <c r="C11" s="1">
-        <v>0.26</v>
+        <v>0.64</v>
       </c>
       <c r="D11" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.22</v>
       </c>
       <c r="E11" s="1">
-        <v>0.18</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1296,13 +2713,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="1">
-        <v>0.3</v>
+        <v>0.62</v>
       </c>
       <c r="D12" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.24</v>
       </c>
       <c r="E12" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1313,13 +2730,13 @@
         <v>46</v>
       </c>
       <c r="C13" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E13" s="1">
         <v>0.13</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0.71</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.16</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1330,13 +2747,13 @@
         <v>19</v>
       </c>
       <c r="C14" s="1">
-        <v>0.16</v>
+        <v>0.67</v>
       </c>
       <c r="D14" s="1">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="E14" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1347,13 +2764,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="1">
-        <v>0.24</v>
+        <v>0.63</v>
       </c>
       <c r="D15" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.23</v>
       </c>
       <c r="E15" s="1">
-        <v>0.19</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1364,13 +2781,13 @@
         <v>12</v>
       </c>
       <c r="C16" s="1">
-        <v>0.2</v>
+        <v>0.63</v>
       </c>
       <c r="D16" s="1">
-        <v>0.66</v>
+        <v>0.24</v>
       </c>
       <c r="E16" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1381,13 +2798,13 @@
         <v>47</v>
       </c>
       <c r="C17" s="1">
-        <v>0.11</v>
+        <v>0.68</v>
       </c>
       <c r="D17" s="1">
-        <v>0.77</v>
+        <v>0.19</v>
       </c>
       <c r="E17" s="1">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1398,13 +2815,13 @@
         <v>41</v>
       </c>
       <c r="C18" s="1">
-        <v>0.11</v>
+        <v>0.67</v>
       </c>
       <c r="D18" s="1">
-        <v>0.77</v>
+        <v>0.19</v>
       </c>
       <c r="E18" s="1">
-        <v>0.12</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1415,13 +2832,13 @@
         <v>10</v>
       </c>
       <c r="C19" s="1">
-        <v>0.21</v>
+        <v>0.65</v>
       </c>
       <c r="D19" s="1">
-        <v>0.68</v>
+        <v>0.22</v>
       </c>
       <c r="E19" s="1">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1432,13 +2849,13 @@
         <v>25</v>
       </c>
       <c r="C20" s="1">
-        <v>0.15</v>
+        <v>0.68</v>
       </c>
       <c r="D20" s="1">
-        <v>0.74</v>
+        <v>0.2</v>
       </c>
       <c r="E20" s="1">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1449,13 +2866,13 @@
         <v>40</v>
       </c>
       <c r="C21" s="1">
-        <v>0.16</v>
+        <v>0.7</v>
       </c>
       <c r="D21" s="1">
-        <v>0.69</v>
+        <v>0.17</v>
       </c>
       <c r="E21" s="1">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1466,13 +2883,13 @@
         <v>8</v>
       </c>
       <c r="C22" s="1">
-        <v>0.34</v>
+        <v>0.62</v>
       </c>
       <c r="D22" s="1">
-        <v>0.47</v>
+        <v>0.23</v>
       </c>
       <c r="E22" s="1">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1483,13 +2900,13 @@
         <v>28</v>
       </c>
       <c r="C23" s="1">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="D23" s="1">
-        <v>0.51</v>
+        <v>0.21</v>
       </c>
       <c r="E23" s="1">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1500,13 +2917,13 @@
         <v>26</v>
       </c>
       <c r="C24" s="1">
-        <v>0.18</v>
+        <v>0.66</v>
       </c>
       <c r="D24" s="1">
-        <v>0.66</v>
+        <v>0.21</v>
       </c>
       <c r="E24" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1517,13 +2934,13 @@
         <v>49</v>
       </c>
       <c r="C25" s="1">
-        <v>0.11</v>
+        <v>0.67</v>
       </c>
       <c r="D25" s="1">
-        <v>0.74</v>
+        <v>0.19</v>
       </c>
       <c r="E25" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1534,10 +2951,10 @@
         <v>14</v>
       </c>
       <c r="C26" s="1">
-        <v>0.17</v>
+        <v>0.69</v>
       </c>
       <c r="D26" s="1">
-        <v>0.72</v>
+        <v>0.2</v>
       </c>
       <c r="E26" s="1">
         <v>0.11</v>
@@ -1551,13 +2968,13 @@
         <v>38</v>
       </c>
       <c r="C27" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.19</v>
+      </c>
+      <c r="E27" s="1">
         <v>0.14000000000000001</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0.74</v>
-      </c>
-      <c r="E27" s="1">
-        <v>0.12</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1568,13 +2985,13 @@
         <v>36</v>
       </c>
       <c r="C28" s="1">
-        <v>0.13</v>
+        <v>0.75</v>
       </c>
       <c r="D28" s="1">
-        <v>0.74</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E28" s="1">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1585,10 +3002,10 @@
         <v>45</v>
       </c>
       <c r="C29" s="1">
-        <v>0.1</v>
+        <v>0.71</v>
       </c>
       <c r="D29" s="1">
-        <v>0.78</v>
+        <v>0.17</v>
       </c>
       <c r="E29" s="1">
         <v>0.12</v>
@@ -1602,13 +3019,13 @@
         <v>32</v>
       </c>
       <c r="C30" s="1">
-        <v>0.19</v>
+        <v>0.65</v>
       </c>
       <c r="D30" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="E30" s="1">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1619,13 +3036,13 @@
         <v>23</v>
       </c>
       <c r="C31" s="1">
-        <v>0.22</v>
+        <v>0.65</v>
       </c>
       <c r="D31" s="1">
-        <v>0.57999999999999996</v>
+        <v>0.21</v>
       </c>
       <c r="E31" s="1">
-        <v>0.2</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1636,13 +3053,13 @@
         <v>16</v>
       </c>
       <c r="C32" s="1">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="D32" s="1">
-        <v>0.47</v>
+        <v>0.23</v>
       </c>
       <c r="E32" s="1">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1653,13 +3070,13 @@
         <v>44</v>
       </c>
       <c r="C33" s="1">
-        <v>0.15</v>
+        <v>0.65</v>
       </c>
       <c r="D33" s="1">
-        <v>0.67</v>
+        <v>0.21</v>
       </c>
       <c r="E33" s="1">
-        <v>0.18</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1670,13 +3087,13 @@
         <v>30</v>
       </c>
       <c r="C34" s="1">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="D34" s="1">
-        <v>0.49</v>
+        <v>0.21</v>
       </c>
       <c r="E34" s="1">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1687,13 +3104,13 @@
         <v>1</v>
       </c>
       <c r="C35" s="1">
-        <v>0.3</v>
+        <v>0.63</v>
       </c>
       <c r="D35" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.24</v>
       </c>
       <c r="E35" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1704,10 +3121,10 @@
         <v>51</v>
       </c>
       <c r="C36" s="1">
-        <v>0.09</v>
+        <v>0.69</v>
       </c>
       <c r="D36" s="1">
-        <v>0.79</v>
+        <v>0.19</v>
       </c>
       <c r="E36" s="1">
         <v>0.12</v>
@@ -1721,13 +3138,13 @@
         <v>15</v>
       </c>
       <c r="C37" s="1">
-        <v>0.21</v>
+        <v>0.63</v>
       </c>
       <c r="D37" s="1">
-        <v>0.64</v>
+        <v>0.23</v>
       </c>
       <c r="E37" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1738,10 +3155,10 @@
         <v>42</v>
       </c>
       <c r="C38" s="1">
-        <v>0.11</v>
+        <v>0.69</v>
       </c>
       <c r="D38" s="1">
-        <v>0.78</v>
+        <v>0.2</v>
       </c>
       <c r="E38" s="1">
         <v>0.11</v>
@@ -1755,13 +3172,13 @@
         <v>22</v>
       </c>
       <c r="C39" s="1">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
       <c r="D39" s="1">
-        <v>0.63</v>
+        <v>0.18</v>
       </c>
       <c r="E39" s="1">
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1772,13 +3189,13 @@
         <v>5</v>
       </c>
       <c r="C40" s="1">
-        <v>0.31</v>
+        <v>0.62</v>
       </c>
       <c r="D40" s="1">
-        <v>0.51</v>
+        <v>0.23</v>
       </c>
       <c r="E40" s="1">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1789,13 +3206,13 @@
         <v>33</v>
       </c>
       <c r="C41" s="1">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="D41" s="1">
-        <v>0.52</v>
+        <v>0.23</v>
       </c>
       <c r="E41" s="1">
-        <v>0.24</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1806,13 +3223,13 @@
         <v>2</v>
       </c>
       <c r="C42" s="1">
-        <v>0.26</v>
+        <v>0.67</v>
       </c>
       <c r="D42" s="1">
-        <v>0.64</v>
+        <v>0.22</v>
       </c>
       <c r="E42" s="1">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1823,13 +3240,13 @@
         <v>50</v>
       </c>
       <c r="C43" s="1">
-        <v>0.09</v>
+        <v>0.76</v>
       </c>
       <c r="D43" s="1">
-        <v>0.8</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E43" s="1">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1840,13 +3257,13 @@
         <v>4</v>
       </c>
       <c r="C44" s="1">
-        <v>0.27</v>
+        <v>0.67</v>
       </c>
       <c r="D44" s="1">
-        <v>0.6</v>
+        <v>0.21</v>
       </c>
       <c r="E44" s="1">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1857,13 +3274,13 @@
         <v>31</v>
       </c>
       <c r="C45" s="1">
-        <v>0.19</v>
+        <v>0.67</v>
       </c>
       <c r="D45" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="E45" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1874,13 +3291,13 @@
         <v>21</v>
       </c>
       <c r="C46" s="1">
-        <v>0.19</v>
+        <v>0.65</v>
       </c>
       <c r="D46" s="1">
-        <v>0.66</v>
+        <v>0.21</v>
       </c>
       <c r="E46" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1891,13 +3308,13 @@
         <v>39</v>
       </c>
       <c r="C47" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="D47" s="1">
         <v>0.18</v>
       </c>
-      <c r="D47" s="1">
-        <v>0.64</v>
-      </c>
       <c r="E47" s="1">
-        <v>0.18</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1908,13 +3325,13 @@
         <v>7</v>
       </c>
       <c r="C48" s="1">
-        <v>0.3</v>
+        <v>0.64</v>
       </c>
       <c r="D48" s="1">
-        <v>0.53</v>
+        <v>0.22</v>
       </c>
       <c r="E48" s="1">
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1925,13 +3342,13 @@
         <v>17</v>
       </c>
       <c r="C49" s="1">
-        <v>0.22</v>
+        <v>0.67</v>
       </c>
       <c r="D49" s="1">
-        <v>0.6</v>
+        <v>0.19</v>
       </c>
       <c r="E49" s="1">
-        <v>0.18</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1942,10 +3359,10 @@
         <v>9</v>
       </c>
       <c r="C50" s="1">
-        <v>0.22</v>
+        <v>0.64</v>
       </c>
       <c r="D50" s="1">
-        <v>0.66</v>
+        <v>0.24</v>
       </c>
       <c r="E50" s="1">
         <v>0.12</v>
@@ -1959,13 +3376,13 @@
         <v>48</v>
       </c>
       <c r="C51" s="1">
-        <v>0.12</v>
+        <v>0.66</v>
       </c>
       <c r="D51" s="1">
-        <v>0.73</v>
+        <v>0.2</v>
       </c>
       <c r="E51" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1976,13 +3393,13 @@
         <v>43</v>
       </c>
       <c r="C52" s="1">
-        <v>0.11</v>
+        <v>0.71</v>
       </c>
       <c r="D52" s="1">
-        <v>0.78</v>
+        <v>0.16</v>
       </c>
       <c r="E52" s="1">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
     </row>
   </sheetData>
@@ -2160,318 +3577,318 @@
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1">
-        <v>0.23</v>
+        <v>0.65</v>
       </c>
       <c r="C2" s="1">
-        <v>0.16</v>
+        <v>0.72</v>
       </c>
       <c r="D2" s="1">
-        <v>0.19</v>
+        <v>0.67</v>
       </c>
       <c r="E2" s="1">
-        <v>0.15</v>
+        <v>0.67</v>
       </c>
       <c r="F2" s="1">
-        <v>0.21</v>
+        <v>0.62</v>
       </c>
       <c r="G2" s="1">
-        <v>0.16</v>
+        <v>0.68</v>
       </c>
       <c r="H2" s="1">
-        <v>0.24</v>
+        <v>0.65</v>
       </c>
       <c r="I2" s="1">
-        <v>0.3</v>
+        <v>0.62</v>
       </c>
       <c r="J2" s="1">
-        <v>0.27</v>
+        <v>0.67</v>
       </c>
       <c r="K2" s="1">
-        <v>0.26</v>
+        <v>0.64</v>
       </c>
       <c r="L2" s="1">
-        <v>0.3</v>
+        <v>0.62</v>
       </c>
       <c r="M2" s="1">
-        <v>0.13</v>
+        <v>0.73</v>
       </c>
       <c r="N2" s="1">
-        <v>0.16</v>
+        <v>0.67</v>
       </c>
       <c r="O2" s="1">
-        <v>0.24</v>
+        <v>0.63</v>
       </c>
       <c r="P2" s="1">
-        <v>0.2</v>
+        <v>0.63</v>
       </c>
       <c r="Q2" s="1">
-        <v>0.11</v>
+        <v>0.68</v>
       </c>
       <c r="R2" s="1">
-        <v>0.11</v>
+        <v>0.67</v>
       </c>
       <c r="S2" s="1">
-        <v>0.21</v>
+        <v>0.65</v>
       </c>
       <c r="T2" s="1">
-        <v>0.15</v>
+        <v>0.68</v>
       </c>
       <c r="U2" s="1">
-        <v>0.16</v>
+        <v>0.7</v>
       </c>
       <c r="V2" s="1">
-        <v>0.34</v>
+        <v>0.62</v>
       </c>
       <c r="W2" s="1">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="X2" s="1">
-        <v>0.18</v>
+        <v>0.66</v>
       </c>
       <c r="Y2" s="1">
-        <v>0.11</v>
+        <v>0.67</v>
       </c>
       <c r="Z2" s="1">
-        <v>0.17</v>
+        <v>0.69</v>
       </c>
       <c r="AA2" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.67</v>
       </c>
       <c r="AB2" s="1">
-        <v>0.13</v>
+        <v>0.75</v>
       </c>
       <c r="AC2" s="1">
-        <v>0.1</v>
+        <v>0.71</v>
       </c>
       <c r="AD2" s="1">
-        <v>0.19</v>
+        <v>0.65</v>
       </c>
       <c r="AE2" s="1">
-        <v>0.22</v>
+        <v>0.65</v>
       </c>
       <c r="AF2" s="1">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="AG2" s="1">
-        <v>0.15</v>
+        <v>0.65</v>
       </c>
       <c r="AH2" s="1">
-        <v>0.24</v>
+        <v>0.62</v>
       </c>
       <c r="AI2" s="1">
-        <v>0.3</v>
+        <v>0.63</v>
       </c>
       <c r="AJ2" s="1">
-        <v>0.09</v>
+        <v>0.69</v>
       </c>
       <c r="AK2" s="1">
-        <v>0.21</v>
+        <v>0.63</v>
       </c>
       <c r="AL2" s="1">
-        <v>0.11</v>
+        <v>0.69</v>
       </c>
       <c r="AM2" s="1">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
       <c r="AN2" s="1">
-        <v>0.31</v>
+        <v>0.62</v>
       </c>
       <c r="AO2" s="1">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="AP2" s="1">
-        <v>0.26</v>
+        <v>0.67</v>
       </c>
       <c r="AQ2" s="1">
-        <v>0.09</v>
+        <v>0.76</v>
       </c>
       <c r="AR2" s="1">
-        <v>0.27</v>
+        <v>0.67</v>
       </c>
       <c r="AS2" s="1">
-        <v>0.19</v>
+        <v>0.67</v>
       </c>
       <c r="AT2" s="1">
-        <v>0.19</v>
+        <v>0.65</v>
       </c>
       <c r="AU2" s="1">
-        <v>0.18</v>
+        <v>0.68</v>
       </c>
       <c r="AV2" s="1">
-        <v>0.3</v>
+        <v>0.64</v>
       </c>
       <c r="AW2" s="1">
-        <v>0.22</v>
+        <v>0.67</v>
       </c>
       <c r="AX2" s="1">
-        <v>0.22</v>
+        <v>0.64</v>
       </c>
       <c r="AY2" s="1">
-        <v>0.12</v>
+        <v>0.66</v>
       </c>
       <c r="AZ2" s="1">
-        <v>0.11</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" s="1">
-        <v>0.68</v>
+        <v>0.23</v>
       </c>
       <c r="C3" s="1">
-        <v>0.64</v>
+        <v>0.15</v>
       </c>
       <c r="D3" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="E3" s="1">
-        <v>0.73</v>
+        <v>0.21</v>
       </c>
       <c r="F3" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.2</v>
       </c>
       <c r="G3" s="1">
-        <v>0.67</v>
+        <v>0.18</v>
       </c>
       <c r="H3" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.21</v>
       </c>
       <c r="I3" s="1">
-        <v>0.51</v>
+        <v>0.25</v>
       </c>
       <c r="J3" s="1">
-        <v>0.41</v>
+        <v>0.17</v>
       </c>
       <c r="K3" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.22</v>
       </c>
       <c r="L3" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.24</v>
       </c>
       <c r="M3" s="1">
-        <v>0.71</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="N3" s="1">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="O3" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.23</v>
       </c>
       <c r="P3" s="1">
-        <v>0.66</v>
+        <v>0.24</v>
       </c>
       <c r="Q3" s="1">
-        <v>0.77</v>
+        <v>0.19</v>
       </c>
       <c r="R3" s="1">
-        <v>0.77</v>
+        <v>0.19</v>
       </c>
       <c r="S3" s="1">
-        <v>0.68</v>
+        <v>0.22</v>
       </c>
       <c r="T3" s="1">
-        <v>0.74</v>
+        <v>0.2</v>
       </c>
       <c r="U3" s="1">
-        <v>0.69</v>
+        <v>0.17</v>
       </c>
       <c r="V3" s="1">
-        <v>0.47</v>
+        <v>0.23</v>
       </c>
       <c r="W3" s="1">
-        <v>0.51</v>
+        <v>0.21</v>
       </c>
       <c r="X3" s="1">
-        <v>0.66</v>
+        <v>0.21</v>
       </c>
       <c r="Y3" s="1">
-        <v>0.74</v>
+        <v>0.19</v>
       </c>
       <c r="Z3" s="1">
-        <v>0.72</v>
+        <v>0.2</v>
       </c>
       <c r="AA3" s="1">
-        <v>0.74</v>
+        <v>0.19</v>
       </c>
       <c r="AB3" s="1">
-        <v>0.74</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="AC3" s="1">
-        <v>0.78</v>
+        <v>0.17</v>
       </c>
       <c r="AD3" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="AE3" s="1">
-        <v>0.57999999999999996</v>
+        <v>0.21</v>
       </c>
       <c r="AF3" s="1">
-        <v>0.47</v>
+        <v>0.23</v>
       </c>
       <c r="AG3" s="1">
-        <v>0.67</v>
+        <v>0.21</v>
       </c>
       <c r="AH3" s="1">
-        <v>0.49</v>
+        <v>0.21</v>
       </c>
       <c r="AI3" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.24</v>
       </c>
       <c r="AJ3" s="1">
-        <v>0.79</v>
+        <v>0.19</v>
       </c>
       <c r="AK3" s="1">
-        <v>0.64</v>
+        <v>0.23</v>
       </c>
       <c r="AL3" s="1">
-        <v>0.78</v>
+        <v>0.2</v>
       </c>
       <c r="AM3" s="1">
-        <v>0.63</v>
+        <v>0.18</v>
       </c>
       <c r="AN3" s="1">
-        <v>0.51</v>
+        <v>0.23</v>
       </c>
       <c r="AO3" s="1">
-        <v>0.52</v>
+        <v>0.23</v>
       </c>
       <c r="AP3" s="1">
-        <v>0.64</v>
+        <v>0.22</v>
       </c>
       <c r="AQ3" s="1">
-        <v>0.8</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="AR3" s="1">
-        <v>0.6</v>
+        <v>0.21</v>
       </c>
       <c r="AS3" s="1">
-        <v>0.65</v>
+        <v>0.2</v>
       </c>
       <c r="AT3" s="1">
-        <v>0.66</v>
+        <v>0.21</v>
       </c>
       <c r="AU3" s="1">
-        <v>0.64</v>
+        <v>0.18</v>
       </c>
       <c r="AV3" s="1">
-        <v>0.53</v>
+        <v>0.22</v>
       </c>
       <c r="AW3" s="1">
-        <v>0.6</v>
+        <v>0.19</v>
       </c>
       <c r="AX3" s="1">
-        <v>0.66</v>
+        <v>0.24</v>
       </c>
       <c r="AY3" s="1">
-        <v>0.73</v>
+        <v>0.2</v>
       </c>
       <c r="AZ3" s="1">
-        <v>0.78</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="4" spans="1:52" x14ac:dyDescent="0.25">
@@ -2634,6 +4051,336 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7710D8-82BE-4E00-AB90-DD20512A3B95}">
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="3">
+        <f>VLOOKUP('sales region lookup'!A2, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.67</v>
+      </c>
+      <c r="D2" s="3">
+        <f>_xlfn.XLOOKUP(A2, 'by search term'!B1:B52, 'by search term'!D1:D52, "not found")</f>
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="3">
+        <f>VLOOKUP('sales region lookup'!A3, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.68</v>
+      </c>
+      <c r="D3" s="3">
+        <f>_xlfn.XLOOKUP(A3, 'by search term'!B2:B53, 'by search term'!D2:D53, "not found")</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="3">
+        <f>VLOOKUP('sales region lookup'!A4, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.67</v>
+      </c>
+      <c r="D4" s="3">
+        <f>_xlfn.XLOOKUP(A4, 'by search term'!B3:B54, 'by search term'!D3:D54, "not found")</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="3">
+        <f>VLOOKUP('sales region lookup'!A5, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.75</v>
+      </c>
+      <c r="D5" s="3">
+        <f>_xlfn.XLOOKUP(A5, 'by search term'!B4:B55, 'by search term'!D4:D55, "not found")</f>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="3">
+        <f>VLOOKUP('sales region lookup'!A6, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.69</v>
+      </c>
+      <c r="D6" s="3">
+        <f>_xlfn.XLOOKUP(A6, 'by search term'!B5:B56, 'by search term'!D5:D56, "not found")</f>
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="3">
+        <f>VLOOKUP('sales region lookup'!A7, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.76</v>
+      </c>
+      <c r="D7" s="3">
+        <f>_xlfn.XLOOKUP(A7, 'by search term'!B6:B57, 'by search term'!D6:D57, "not found")</f>
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="3">
+        <f>VLOOKUP('sales region lookup'!A8, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.71</v>
+      </c>
+      <c r="D8" s="3">
+        <f>_xlfn.XLOOKUP(A8, 'by search term'!B7:B58, 'by search term'!D7:D58, "not found")</f>
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="3">
+        <f>VLOOKUP('sales region lookup'!A9, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.67</v>
+      </c>
+      <c r="D9" s="3">
+        <f>_xlfn.XLOOKUP(A9, 'by search term'!B8:B59, 'by search term'!D8:D59, "not found")</f>
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="3">
+        <f>VLOOKUP('sales region lookup'!A10, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.66</v>
+      </c>
+      <c r="D10" s="3">
+        <f>_xlfn.XLOOKUP(A10, 'by search term'!B9:B60, 'by search term'!D9:D60, "not found")</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="3">
+        <f>VLOOKUP('sales region lookup'!A11, 'by search term'!B:D, 2, FALSE)</f>
+        <v>0.66</v>
+      </c>
+      <c r="D11" s="3">
+        <f>_xlfn.XLOOKUP(A11, 'by search term'!B10:B61, 'by search term'!D10:D61, "not found")</f>
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0.71</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="1">
+        <v>0.76</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0.67</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="1">
+        <v>6.92</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1.8099999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>